<commit_message>
Split the floor guard from the remediation record in the storyboard
The workbook still credited varRemediationFlag with guarding the accumulation
floor, while the same variable is deliberately preserved across Retry so the
recovery layer and the LMS record survive. One variable cannot do both jobs: on
every attempt after the first the floor would never fire, and a learner could
accumulate to 30 without being stopped once.

varFloorFired is the guard and resets with the attempt. varRemediationFlag is the
record and does not. The categorical gate sits behind neither — it is guarded per
decision point, because a learner stopped at DP1 must still be stopped when they
choose to enter the dwelling at DP4.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JLHR8zxTnU1oW4Rgc2RYK4
</commit_message>
<xml_diff>
--- a/public/first-15/production-storyboard.xlsx
+++ b/public/first-15/production-storyboard.xlsx
@@ -1242,7 +1242,7 @@
     <t xml:space="preserve">Adjust variable varSafetyScore - subtract the option's authored cost (20 at DP1, 25 at DP4)</t>
   </si>
   <si>
-    <t xml:space="preserve">The flag guard, not a restore value, prevents the infinite re-trap: varRemediationFlag = True blocks the floor trigger for the rest of the attempt, so the score is free to stay low.</t>
+    <t xml:space="preserve">The guard, not a restore value, prevents the infinite re-trap: varFloorFired = True blocks the floor trigger for the rest of the attempt, so the score is free to stay low. Keep this separate from varRemediationFlag, which is the record and survives Retry - if one variable does both jobs, the floor never fires again after the first attempt.</t>
   </si>
   <si>
     <t xml:space="preserve">Change state of btnDPn_&lt;critical option&gt; to Disabled</t>
@@ -1371,7 +1371,7 @@
     <t xml:space="preserve">After the micro-lesson the learner returns to the decision with Safety still at 50. Re-deciding DP1 with option B (−10) lands at 40, which trips the floor again — forever.</t>
   </si>
   <si>
-    <t xml:space="preserve">Two changes: apply the chosen option's authored Safety cost at the end of the micro-lesson and clamp to 0-100 - NOT a flat restore to 60. A flat restore hands points to any learner who reached the gate already below 60, so the gate rewards the violation it exists to punish; a gate that can raise your score is not a gate. AND guard the floor trigger with varRemediationFlag = False so it fires at most once per attempt. The guard is what prevents the re-trap, which is why the score no longer has to be propped up.</t>
+    <t xml:space="preserve">Two changes: apply the chosen option's authored Safety cost at the end of the micro-lesson and clamp to 0-100 - NOT a flat restore to 60. A flat restore hands points to any learner who reached the gate already below 60, so the gate rewards the violation it exists to punish; a gate that can raise your score is not a gate. AND guard the floor trigger with varFloorFired = False so it fires at most once per attempt. The guard is what prevents the re-trap, which is why the score no longer has to be propped up. The categorical gate (1C, 4B) is NOT behind that guard - it is guarded per decision point, or a learner stopped once at DP1 walks into the dwelling at DP4 unchallenged.</t>
   </si>
   <si>
     <t xml:space="preserve">A second attempt produces impossible scores.</t>

</xml_diff>